<commit_message>
release: prepare V1.6.17 instruction and runtime update
</commit_message>
<xml_diff>
--- a/skills/high-tech-enterprise-preassessment/assets/高企预评估双年度采集表.xlsx
+++ b/skills/high-tech-enterprise-preassessment/assets/高企预评估双年度采集表.xlsx
@@ -12,6 +12,26 @@
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="补强计划" sheetId="8" r:id="R8078999a7d864d64"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规则与来源" sheetId="9" r:id="R38177643c9c84a74"/>
   </x:sheets>
+  <x:definedNames>
+    <x:definedName name="_xlnm.Print_Area" localSheetId="0">'使用说明'!$A$1:$H$20</x:definedName>
+    <x:definedName name="_xlnm.Print_Titles" localSheetId="0">'使用说明'!$4:$4</x:definedName>
+    <x:definedName name="_xlnm.Print_Area" localSheetId="1">'基础与硬门槛'!$A$1:$F$26</x:definedName>
+    <x:definedName name="_xlnm.Print_Titles" localSheetId="1">'基础与硬门槛'!$4:$4</x:definedName>
+    <x:definedName name="_xlnm.Print_Area" localSheetId="2">'财务与成长性'!$A$1:$H$26</x:definedName>
+    <x:definedName name="_xlnm.Print_Titles" localSheetId="2">'财务与成长性'!$4:$4</x:definedName>
+    <x:definedName name="_xlnm.Print_Area" localSheetId="3">'知识产权'!$A$1:$S$104</x:definedName>
+    <x:definedName name="_xlnm.Print_Titles" localSheetId="3">'知识产权'!$4:$4</x:definedName>
+    <x:definedName name="_xlnm.Print_Area" localSheetId="4">'成果转化'!$A$1:$P$104</x:definedName>
+    <x:definedName name="_xlnm.Print_Titles" localSheetId="4">'成果转化'!$4:$4</x:definedName>
+    <x:definedName name="_xlnm.Print_Area" localSheetId="5">'组织管理'!$A$1:$K$22</x:definedName>
+    <x:definedName name="_xlnm.Print_Titles" localSheetId="5">'组织管理'!$4:$4</x:definedName>
+    <x:definedName name="_xlnm.Print_Area" localSheetId="6">'双年度评分'!$A$1:$J$18</x:definedName>
+    <x:definedName name="_xlnm.Print_Titles" localSheetId="6">'双年度评分'!$4:$4</x:definedName>
+    <x:definedName name="_xlnm.Print_Area" localSheetId="7">'补强计划'!$A$1:$K$64</x:definedName>
+    <x:definedName name="_xlnm.Print_Titles" localSheetId="7">'补强计划'!$4:$4</x:definedName>
+    <x:definedName name="_xlnm.Print_Area" localSheetId="8">'规则与来源'!$A$1:$F$14</x:definedName>
+    <x:definedName name="_xlnm.Print_Titles" localSheetId="8">'规则与来源'!$4:$4</x:definedName>
+  </x:definedNames>
 </x:workbook>
 </file>
 
@@ -668,6 +688,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:pageSetUpPr fitToPage="1" autoPageBreaks="0"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="9" hidden="0" customWidth="1"/>
@@ -1179,12 +1202,16 @@
       <x:formula1>"未开始,进行中,已完成,不适用"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.3" footer="0.3"/>
+  <x:pageSetup orientation="landscape" paperSize="9" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:pageSetUpPr fitToPage="1" autoPageBreaks="0"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="9" hidden="0" customWidth="1"/>
@@ -1575,12 +1602,16 @@
       <x:formula1>"是,否,待核"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.3" footer="0.3"/>
+  <x:pageSetup orientation="landscape" paperSize="9" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:pageSetUpPr fitToPage="1" autoPageBreaks="0"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
@@ -2152,12 +2183,16 @@
     <x:mergeCell ref="A16:H16"/>
     <x:mergeCell ref="A23:H23"/>
   </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.3" footer="0.3"/>
+  <x:pageSetup orientation="landscape" paperSize="9" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:pageSetUpPr fitToPage="1" autoPageBreaks="0"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
@@ -5314,7 +5349,8 @@
       <x:formula1>"完整,部分,薄弱,待核"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.3" footer="0.3"/>
+  <x:pageSetup orientation="landscape" paperSize="8" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver"/>
   <x:tableParts count="1">
     <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76ed40c6bbae47ee"/>
   </x:tableParts>
@@ -5323,6 +5359,9 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:pageSetUpPr fitToPage="1" autoPageBreaks="0"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
@@ -8432,7 +8471,8 @@
       <x:formula1>"是,否,待核"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.3" footer="0.3"/>
+  <x:pageSetup orientation="landscape" paperSize="8" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver"/>
   <x:tableParts count="1">
     <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49ff1b2fc68e4c05"/>
   </x:tableParts>
@@ -8441,6 +8481,9 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:pageSetUpPr fitToPage="1" autoPageBreaks="0"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
@@ -8968,12 +9011,16 @@
       <x:formula1>"证据补强,事实补强,无缺口,待核"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.3" footer="0.3"/>
+  <x:pageSetup orientation="landscape" paperSize="8" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:pageSetUpPr fitToPage="1" autoPageBreaks="0"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
@@ -9472,12 +9519,16 @@
       <x:formula2>30</x:formula2>
     </x:dataValidation>
   </x:dataValidations>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.3" footer="0.3"/>
+  <x:pageSetup orientation="landscape" paperSize="8" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:pageSetUpPr fitToPage="1" autoPageBreaks="0"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
@@ -10767,7 +10818,8 @@
       <x:formula1>"未开始,进行中,已完成,不适用"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.3" footer="0.3"/>
+  <x:pageSetup orientation="landscape" paperSize="8" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver"/>
   <x:tableParts count="1">
     <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1d0a2d8da464016"/>
   </x:tableParts>
@@ -10776,6 +10828,9 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:pageSetUpPr fitToPage="1" autoPageBreaks="0"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
@@ -11059,6 +11114,7 @@
     <x:mergeCell ref="A1:F1"/>
     <x:mergeCell ref="A2:F2"/>
   </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.3" footer="0.3"/>
+  <x:pageSetup orientation="landscape" paperSize="9" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver"/>
 </x:worksheet>
 </file>
</xml_diff>